<commit_message>
CORE-000216 edit: added TMRPT to output variables
</commit_message>
<xml_diff>
--- a/rules/CORE-000216/negative/01/data/unit-test-coreid-CG0545-negative 1.xlsx
+++ b/rules/CORE-000216/negative/01/data/unit-test-coreid-CG0545-negative 1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marisa_wyckmans\CORE\CDISC_Rule_Authoring\core-contributor\rules\CORE-000216\negative\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6012AB12-15FD-42F5-A931-233F68F6EAE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0518FD0E-A043-4BEA-AA1A-17CD6911B466}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="555" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="555" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="55">
   <si>
     <t>Product</t>
   </si>
@@ -638,7 +638,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="15.5703125" customWidth="1"/>
@@ -687,22 +687,62 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C3" t="s">
         <v>54</v>
       </c>
       <c r="D3">
+        <v>5</v>
+      </c>
+      <c r="E3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D4">
         <v>6</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E4" t="s">
         <v>18</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F4" t="s">
         <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" t="s">
+        <v>54</v>
+      </c>
+      <c r="D5">
+        <v>5</v>
+      </c>
+      <c r="E5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -796,7 +836,7 @@
       <c r="D5" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="5" t="s">
         <v>31</v>
       </c>
     </row>

</xml_diff>